<commit_message>
docs: refresh migration manifest (193 tracked files)
Regenerated from the current git-tracked set — adds everything shipped
since the last manifest: trust-layer services (replay, agent_health,
challenger, evals, pipeline_view), eval golden data (new mandatory
category — the test suite fails without it), prompts v3-v5, new tests,
PipelineGraph, SEVERITY.md. The manifest itself is marked reference-only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MIGRATION-FILES.xlsx
+++ b/docs/MIGRATION-FILES.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Rebuild steps" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Files to migrate'!$A$1:$E$178</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Files to migrate'!$A$1:$E$194</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E178"/>
+  <dimension ref="A1:E194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/artifacts/__init__.py</t>
+          <t>backend/app/services/agent_health.py</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/artifacts/parsers.py</t>
+          <t>backend/app/services/artifacts/__init__.py</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/artifacts/service.py</t>
+          <t>backend/app/services/artifacts/parsers.py</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -1687,7 +1687,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/audit.py</t>
+          <t>backend/app/services/artifacts/service.py</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/copado/__init__.py</t>
+          <t>backend/app/services/audit.py</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/copado/fixtures.py</t>
+          <t>backend/app/services/challenger.py</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/copado/normaliser.py</t>
+          <t>backend/app/services/copado/__init__.py</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/copado/service.py</t>
+          <t>backend/app/services/copado/fixtures.py</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/evidence_pack.py</t>
+          <t>backend/app/services/copado/normaliser.py</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/feedback.py</t>
+          <t>backend/app/services/copado/service.py</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/github/__init__.py</t>
+          <t>backend/app/services/evals.py</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/github/adapter.py</t>
+          <t>backend/app/services/evidence_pack.py</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/github/factory.py</t>
+          <t>backend/app/services/feedback.py</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/github/mock_adapter.py</t>
+          <t>backend/app/services/github/__init__.py</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/github/rest_adapter.py</t>
+          <t>backend/app/services/github/adapter.py</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/github/service.py</t>
+          <t>backend/app/services/github/factory.py</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -2012,7 +2012,7 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/__init__.py</t>
+          <t>backend/app/services/github/mock_adapter.py</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/adapter.py</t>
+          <t>backend/app/services/github/rest_adapter.py</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/adf.py</t>
+          <t>backend/app/services/github/service.py</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/factory.py</t>
+          <t>backend/app/services/jira/__init__.py</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/field_mapping.py</t>
+          <t>backend/app/services/jira/adapter.py</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/mock_adapter.py</t>
+          <t>backend/app/services/jira/adf.py</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/push_service.py</t>
+          <t>backend/app/services/jira/factory.py</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/rest_adapter.py</t>
+          <t>backend/app/services/jira/field_mapping.py</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/sync_service.py</t>
+          <t>backend/app/services/jira/mock_adapter.py</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/referee.py</t>
+          <t>backend/app/services/jira/push_service.py</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/scheduler.py</t>
+          <t>backend/app/services/jira/rest_adapter.py</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/settings_service.py</t>
+          <t>backend/app/services/jira/sync_service.py</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/work_service.py</t>
+          <t>backend/app/services/pipeline_view.py</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/workflow.py</t>
+          <t>backend/app/services/referee.py</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/ws.py</t>
+          <t>backend/app/services/replay.py</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -2382,12 +2382,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/ac_compliance/v1.md</t>
+          <t>backend/app/services/scheduler.py</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2407,12 +2407,12 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/ac_compliance/v2.md</t>
+          <t>backend/app/services/settings_service.py</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2432,12 +2432,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/ac_compliance/v3.md</t>
+          <t>backend/app/services/work_service.py</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2457,12 +2457,12 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/apex_coverage/v1.md</t>
+          <t>backend/app/services/workflow.py</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2482,12 +2482,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/apex_coverage/v2.md</t>
+          <t>backend/app/services/ws.py</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/apex_coverage/v3.md</t>
+          <t>backend/prompts/ac_compliance/v1.md</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/bdd_generator/v1.md</t>
+          <t>backend/prompts/ac_compliance/v2.md</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/bdd_generator/v2.md</t>
+          <t>backend/prompts/ac_compliance/v3.md</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/bdd_generator/v3.md</t>
+          <t>backend/prompts/apex_coverage/v1.md</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -2612,7 +2612,7 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/change_management/v1.md</t>
+          <t>backend/prompts/apex_coverage/v2.md</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/change_management/v2.md</t>
+          <t>backend/prompts/apex_coverage/v3.md</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/code_review/v1.md</t>
+          <t>backend/prompts/bdd_generator/v1.md</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/code_review/v2.md</t>
+          <t>backend/prompts/bdd_generator/v2.md</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/compliance_ac_advisor/v1.md</t>
+          <t>backend/prompts/bdd_generator/v3.md</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/consumer_duty_mapper/v1.md</t>
+          <t>backend/prompts/bdd_generator/v4.md</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
@@ -2762,7 +2762,7 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/defect_triage/v1.md</t>
+          <t>backend/prompts/change_management/v1.md</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/deployability_validation/v1.md</t>
+          <t>backend/prompts/change_management/v2.md</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/deployment_risk/v1.md</t>
+          <t>backend/prompts/code_review/v1.md</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -2837,7 +2837,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/deployment_risk/v2.md</t>
+          <t>backend/prompts/code_review/v2.md</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/fca_regulatory_impact/v1.md</t>
+          <t>backend/prompts/compliance_ac_advisor/v1.md</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/financial_data_integrity/v1.md</t>
+          <t>backend/prompts/consumer_duty_mapper/v1.md</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/financial_data_integrity/v2.md</t>
+          <t>backend/prompts/defect_triage/v1.md</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/integration_e2e_journey/v1.md</t>
+          <t>backend/prompts/deployability_validation/v1.md</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/monitoring_hypercare/v1.md</t>
+          <t>backend/prompts/deployment_risk/v1.md</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/monitoring_hypercare/v2.md</t>
+          <t>backend/prompts/deployment_risk/v2.md</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
@@ -3012,7 +3012,7 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/post_deploy_verification/v1.md</t>
+          <t>backend/prompts/fca_regulatory_impact/v1.md</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/regression_scope/v1.md</t>
+          <t>backend/prompts/financial_data_integrity/v1.md</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/regression_scope/v2.md</t>
+          <t>backend/prompts/financial_data_integrity/v2.md</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/regulatory_audit_trail/v1.md</t>
+          <t>backend/prompts/integration_e2e_journey/v1.md</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/regulatory_audit_trail/v2.md</t>
+          <t>backend/prompts/monitoring_hypercare/v1.md</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/release_notes/v1.md</t>
+          <t>backend/prompts/monitoring_hypercare/v2.md</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/release_readiness/v1.md</t>
+          <t>backend/prompts/post_deploy_verification/v1.md</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/release_readiness/v2.md</t>
+          <t>backend/prompts/regression_scope/v1.md</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/security_dast/v1.md</t>
+          <t>backend/prompts/regression_scope/v2.md</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/static_analysis/v1.md</t>
+          <t>backend/prompts/regulatory_audit_trail/v1.md</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/static_analysis/v2.md</t>
+          <t>backend/prompts/regulatory_audit_trail/v2.md</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/static_analysis/v3.md</t>
+          <t>backend/prompts/release_notes/v1.md</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/story_quality/v1.md</t>
+          <t>backend/prompts/release_readiness/v1.md</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/test_data_management/v1.md</t>
+          <t>backend/prompts/release_readiness/v2.md</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/test_execution_analyst/v1.md</t>
+          <t>backend/prompts/security_dast/v1.md</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/test_execution_analyst/v2.md</t>
+          <t>backend/prompts/static_analysis/v1.md</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/three_amigos/v1.md</t>
+          <t>backend/prompts/static_analysis/v2.md</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/three_amigos/v2.md</t>
+          <t>backend/prompts/static_analysis/v3.md</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/uat_signoff_coordinator/v1.md</t>
+          <t>backend/prompts/story_quality/v1.md</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/uat_signoff_coordinator/v2.md</t>
+          <t>backend/prompts/test_data_management/v1.md</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
@@ -3507,12 +3507,12 @@
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/__init__.py</t>
+          <t>backend/prompts/test_execution_analyst/v1.md</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -3522,7 +3522,7 @@
       </c>
       <c r="E121" s="6" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3532,12 +3532,12 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/conftest.py</t>
+          <t>backend/prompts/test_execution_analyst/v2.md</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
@@ -3547,7 +3547,7 @@
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3557,12 +3557,12 @@
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_api.py</t>
+          <t>backend/prompts/three_amigos/v1.md</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="E123" s="6" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3582,12 +3582,12 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_artifacts.py</t>
+          <t>backend/prompts/three_amigos/v2.md</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3607,12 +3607,12 @@
       </c>
       <c r="B125" s="5" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_audit.py</t>
+          <t>backend/prompts/three_amigos/v3.md</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
@@ -3622,7 +3622,7 @@
       </c>
       <c r="E125" s="6" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3632,12 +3632,12 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_confidence.py</t>
+          <t>backend/prompts/three_amigos/v4.md</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
@@ -3647,7 +3647,7 @@
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3657,12 +3657,12 @@
       </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_copado.py</t>
+          <t>backend/prompts/three_amigos/v5.md</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
@@ -3672,7 +3672,7 @@
       </c>
       <c r="E127" s="6" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3682,12 +3682,12 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_dev_agents.py</t>
+          <t>backend/prompts/uat_signoff_coordinator/v1.md</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3707,12 +3707,12 @@
       </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_engine.py</t>
+          <t>backend/prompts/uat_signoff_coordinator/v2.md</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="E129" s="6" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3732,12 +3732,12 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Eval golden data</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_evidence_pack.py</t>
+          <t>backend/evals/golden/financial_data_integrity.json</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Expert-labelled golden cases — the test suite (and eval harness) fails without them.</t>
         </is>
       </c>
     </row>
@@ -3762,7 +3762,7 @@
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_feedback.py</t>
+          <t>backend/tests/__init__.py</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_github.py</t>
+          <t>backend/tests/conftest.py</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_push.py</t>
+          <t>backend/tests/test_api.py</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
@@ -3837,7 +3837,7 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_referee.py</t>
+          <t>backend/tests/test_artifacts.py</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
@@ -3862,7 +3862,7 @@
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_refinement_regulatory.py</t>
+          <t>backend/tests/test_audit.py</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_release_agents.py</t>
+          <t>backend/tests/test_confidence.py</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_rest_adapter.py</t>
+          <t>backend/tests/test_copado.py</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
@@ -3937,7 +3937,7 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_settings.py</t>
+          <t>backend/tests/test_dev_agents.py</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_severity.py</t>
+          <t>backend/tests/test_engine.py</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
@@ -3987,7 +3987,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_skip.py</t>
+          <t>backend/tests/test_evidence_pack.py</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_sync.py</t>
+          <t>backend/tests/test_feedback.py</t>
         </is>
       </c>
       <c r="D141" s="3" t="inlineStr">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_testing_agents.py</t>
+          <t>backend/tests/test_github.py</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_traceability.py</t>
+          <t>backend/tests/test_pipeline_view.py</t>
         </is>
       </c>
       <c r="D143" s="3" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_work_queue.py</t>
+          <t>backend/tests/test_push.py</t>
         </is>
       </c>
       <c r="D144" s="3" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_workflow.py</t>
+          <t>backend/tests/test_referee.py</t>
         </is>
       </c>
       <c r="D145" s="3" t="inlineStr">
@@ -4132,12 +4132,12 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Backend (other)</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>backend/pytest.ini</t>
+          <t>backend/tests/test_refinement_regulatory.py</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>Backend support file.</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4157,12 +4157,12 @@
       </c>
       <c r="B147" s="5" t="inlineStr">
         <is>
-          <t>Frontend deps</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>frontend/package-lock.json</t>
+          <t>backend/tests/test_release_agents.py</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="E147" s="6" t="inlineStr">
         <is>
-          <t>npm manifest + lockfile — reproducible install. DO migrate these.</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4182,12 +4182,12 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Frontend deps</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>frontend/package.json</t>
+          <t>backend/tests/test_replay.py</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
@@ -4197,7 +4197,7 @@
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>npm manifest + lockfile — reproducible install. DO migrate these.</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4207,12 +4207,12 @@
       </c>
       <c r="B149" s="5" t="inlineStr">
         <is>
-          <t>Frontend config</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>frontend/index.html</t>
+          <t>backend/tests/test_rest_adapter.py</t>
         </is>
       </c>
       <c r="D149" s="3" t="inlineStr">
@@ -4222,7 +4222,7 @@
       </c>
       <c r="E149" s="6" t="inlineStr">
         <is>
-          <t>Vite/TS/Tailwind/PostCSS config + index.html.</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4232,12 +4232,12 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Frontend config</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>frontend/tsconfig.json</t>
+          <t>backend/tests/test_settings.py</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
@@ -4247,7 +4247,7 @@
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>Vite/TS/Tailwind/PostCSS config + index.html.</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4257,12 +4257,12 @@
       </c>
       <c r="B151" s="5" t="inlineStr">
         <is>
-          <t>Frontend config</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>frontend/vite.config.ts</t>
+          <t>backend/tests/test_severity.py</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E151" s="6" t="inlineStr">
         <is>
-          <t>Vite/TS/Tailwind/PostCSS config + index.html.</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4282,12 +4282,12 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/App.tsx</t>
+          <t>backend/tests/test_skip.py</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
@@ -4297,7 +4297,7 @@
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4307,12 +4307,12 @@
       </c>
       <c r="B153" s="5" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/ErrorBoundary.tsx</t>
+          <t>backend/tests/test_sync.py</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -4322,7 +4322,7 @@
       </c>
       <c r="E153" s="6" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4332,12 +4332,12 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/api.ts</t>
+          <t>backend/tests/test_testing_agents.py</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4357,12 +4357,12 @@
       </c>
       <c r="B155" s="5" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C155" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/components/ArtifactsPanel.tsx</t>
+          <t>backend/tests/test_three_amigos_enrichment.py</t>
         </is>
       </c>
       <c r="D155" s="3" t="inlineStr">
@@ -4372,7 +4372,7 @@
       </c>
       <c r="E155" s="6" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4382,12 +4382,12 @@
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/components/AuditView.tsx</t>
+          <t>backend/tests/test_traceability.py</t>
         </is>
       </c>
       <c r="D156" s="3" t="inlineStr">
@@ -4397,7 +4397,7 @@
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4407,12 +4407,12 @@
       </c>
       <c r="B157" s="5" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C157" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/components/GateModal.tsx</t>
+          <t>backend/tests/test_trust_services.py</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="E157" s="6" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4432,12 +4432,12 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/components/InsightsView.tsx</t>
+          <t>backend/tests/test_work_queue.py</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4457,12 +4457,12 @@
       </c>
       <c r="B159" s="5" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C159" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/components/PipelineBoard.tsx</t>
+          <t>backend/tests/test_workflow.py</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
@@ -4472,7 +4472,7 @@
       </c>
       <c r="E159" s="6" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4482,12 +4482,12 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend (other)</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/components/PushQueueView.tsx</t>
+          <t>backend/pytest.ini</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
@@ -4497,7 +4497,7 @@
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Backend support file.</t>
         </is>
       </c>
     </row>
@@ -4507,12 +4507,12 @@
       </c>
       <c r="B161" s="5" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Frontend deps</t>
         </is>
       </c>
       <c r="C161" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/components/RunCard.tsx</t>
+          <t>frontend/package-lock.json</t>
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="E161" s="6" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>npm manifest + lockfile — reproducible install. DO migrate these.</t>
         </is>
       </c>
     </row>
@@ -4532,12 +4532,12 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Frontend deps</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/components/SettingsPage.tsx</t>
+          <t>frontend/package.json</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
@@ -4547,7 +4547,7 @@
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>npm manifest + lockfile — reproducible install. DO migrate these.</t>
         </is>
       </c>
     </row>
@@ -4557,12 +4557,12 @@
       </c>
       <c r="B163" s="5" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Frontend config</t>
         </is>
       </c>
       <c r="C163" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/components/StoryDrawer.tsx</t>
+          <t>frontend/index.html</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="E163" s="6" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Vite/TS/Tailwind/PostCSS config + index.html.</t>
         </is>
       </c>
     </row>
@@ -4582,12 +4582,12 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Frontend config</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/components/WorkQueue.tsx</t>
+          <t>frontend/tsconfig.json</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Vite/TS/Tailwind/PostCSS config + index.html.</t>
         </is>
       </c>
     </row>
@@ -4607,12 +4607,12 @@
       </c>
       <c r="B165" s="5" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Frontend config</t>
         </is>
       </c>
       <c r="C165" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/index.css</t>
+          <t>frontend/vite.config.ts</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
@@ -4622,7 +4622,7 @@
       </c>
       <c r="E165" s="6" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Vite/TS/Tailwind/PostCSS config + index.html.</t>
         </is>
       </c>
     </row>
@@ -4637,7 +4637,7 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/main.tsx</t>
+          <t>frontend/src/App.tsx</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
@@ -4662,7 +4662,7 @@
       </c>
       <c r="C167" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/types.ts</t>
+          <t>frontend/src/ErrorBoundary.tsx</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -4687,7 +4687,7 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/ui.tsx</t>
+          <t>frontend/src/api.ts</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="C169" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/ws.ts</t>
+          <t>frontend/src/components/ArtifactsPanel.tsx</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
@@ -4732,12 +4732,12 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Frontend (other)</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>frontend/.gitignore</t>
+          <t>frontend/src/components/AuditView.tsx</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -4747,7 +4747,7 @@
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>Frontend support file.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -4757,12 +4757,12 @@
       </c>
       <c r="B171" s="5" t="inlineStr">
         <is>
-          <t>Frontend (other)</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C171" s="5" t="inlineStr">
         <is>
-          <t>frontend/tsconfig.tsbuildinfo</t>
+          <t>frontend/src/components/GateModal.tsx</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
@@ -4772,7 +4772,7 @@
       </c>
       <c r="E171" s="6" t="inlineStr">
         <is>
-          <t>Frontend support file.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -4782,22 +4782,22 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
-        </is>
-      </c>
-      <c r="D172" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/components/InsightsView.tsx</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>Setup + overview. Read before running setup.ps1.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -4807,22 +4807,22 @@
       </c>
       <c r="B173" s="5" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C173" s="5" t="inlineStr">
         <is>
-          <t>docs/COPADO-INTEGRATION.md</t>
-        </is>
-      </c>
-      <c r="D173" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/components/PipelineBoard.tsx</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E173" s="6" t="inlineStr">
         <is>
-          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -4832,22 +4832,22 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>docs/File-Manifest.xlsx</t>
-        </is>
-      </c>
-      <c r="D174" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/components/PipelineGraph.tsx</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -4857,22 +4857,22 @@
       </c>
       <c r="B175" s="5" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C175" s="5" t="inlineStr">
         <is>
-          <t>docs/RESTRICTED-LAPTOP.md</t>
-        </is>
-      </c>
-      <c r="D175" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/components/PushQueueView.tsx</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E175" s="6" t="inlineStr">
         <is>
-          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -4882,22 +4882,22 @@
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>docs/ROADMAP.md</t>
-        </is>
-      </c>
-      <c r="D176" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/components/RunCard.tsx</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -4907,22 +4907,22 @@
       </c>
       <c r="B177" s="5" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C177" s="5" t="inlineStr">
         <is>
-          <t>docs/SEVERITY.md</t>
-        </is>
-      </c>
-      <c r="D177" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/components/SettingsPage.tsx</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E177" s="6" t="inlineStr">
         <is>
-          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -4932,27 +4932,427 @@
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
+          <t>Frontend source</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>frontend/src/components/StoryDrawer.tsx</t>
+        </is>
+      </c>
+      <c r="D178" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E178" s="4" t="inlineStr">
+        <is>
+          <t>React app source (components, types, api client).</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" s="5" t="inlineStr">
+        <is>
+          <t>Frontend source</t>
+        </is>
+      </c>
+      <c r="C179" s="5" t="inlineStr">
+        <is>
+          <t>frontend/src/components/WorkQueue.tsx</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E179" s="6" t="inlineStr">
+        <is>
+          <t>React app source (components, types, api client).</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>Frontend source</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>frontend/src/index.css</t>
+        </is>
+      </c>
+      <c r="D180" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E180" s="4" t="inlineStr">
+        <is>
+          <t>React app source (components, types, api client).</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" s="5" t="inlineStr">
+        <is>
+          <t>Frontend source</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>frontend/src/main.tsx</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E181" s="6" t="inlineStr">
+        <is>
+          <t>React app source (components, types, api client).</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>Frontend source</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>frontend/src/types.ts</t>
+        </is>
+      </c>
+      <c r="D182" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E182" s="4" t="inlineStr">
+        <is>
+          <t>React app source (components, types, api client).</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="5" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" s="5" t="inlineStr">
+        <is>
+          <t>Frontend source</t>
+        </is>
+      </c>
+      <c r="C183" s="5" t="inlineStr">
+        <is>
+          <t>frontend/src/ui.tsx</t>
+        </is>
+      </c>
+      <c r="D183" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E183" s="6" t="inlineStr">
+        <is>
+          <t>React app source (components, types, api client).</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>Frontend source</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>frontend/src/ws.ts</t>
+        </is>
+      </c>
+      <c r="D184" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E184" s="4" t="inlineStr">
+        <is>
+          <t>React app source (components, types, api client).</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>Frontend (other)</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="inlineStr">
+        <is>
+          <t>frontend/.gitignore</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E185" s="6" t="inlineStr">
+        <is>
+          <t>Frontend support file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>Frontend (other)</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>frontend/tsconfig.tsbuildinfo</t>
+        </is>
+      </c>
+      <c r="D186" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E186" s="4" t="inlineStr">
+        <is>
+          <t>Frontend support file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" s="5" t="inlineStr">
+        <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="C178" s="2" t="inlineStr">
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+      <c r="D187" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E187" s="6" t="inlineStr">
+        <is>
+          <t>Setup + overview. Read before running setup.ps1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>docs/COPADO-INTEGRATION.md</t>
+        </is>
+      </c>
+      <c r="D188" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E188" s="4" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>docs/File-Manifest.xlsx</t>
+        </is>
+      </c>
+      <c r="D189" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E189" s="6" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>docs/MIGRATION-FILES.xlsx</t>
+        </is>
+      </c>
+      <c r="D190" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E190" s="4" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>docs/RESTRICTED-LAPTOP.md</t>
+        </is>
+      </c>
+      <c r="D191" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E191" s="6" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>docs/ROADMAP.md</t>
+        </is>
+      </c>
+      <c r="D192" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E192" s="4" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>docs/SEVERITY.md</t>
+        </is>
+      </c>
+      <c r="D193" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E193" s="6" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
         <is>
           <t>docs/Typing-Checklist.xlsx</t>
         </is>
       </c>
-      <c r="D178" s="7" t="inlineStr">
+      <c r="D194" s="7" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="E178" s="4" t="inlineStr">
+      <c r="E194" s="4" t="inlineStr">
         <is>
           <t>Design/spec docs. Not needed to run, needed to understand.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E178"/>
+  <autoFilter ref="A1:E194"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: refresh migration manifest (207 tracked files)
Adds everything since the last manifest: reporting capability
(release/report_snapshot models, reporting service, reports API,
ReportsView), risk register + flaky intelligence (models, services,
APIs, RiskRegisterView), gate-rejection recovery test, and the updated
frontend (App/api/types).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MIGRATION-FILES.xlsx
+++ b/docs/MIGRATION-FILES.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Rebuild steps" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Files to migrate'!$A$1:$E$194</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Files to migrate'!$A$1:$E$208</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E194"/>
+  <dimension ref="A1:E208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>backend/app/api/runs.py</t>
+          <t>backend/app/api/reports.py</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>backend/app/api/settings.py</t>
+          <t>backend/app/api/risk_register.py</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>backend/app/api/stories.py</t>
+          <t>backend/app/api/runs.py</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>backend/app/api/work.py</t>
+          <t>backend/app/api/settings.py</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>backend/app/api/ws.py</t>
+          <t>backend/app/api/stories.py</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1182,12 +1182,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Backend models</t>
+          <t>Backend API</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>backend/app/models/__init__.py</t>
+          <t>backend/app/api/work.py</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>SQLAlchemy ORM / enums — the DB schema.</t>
+          <t>FastAPI routes.</t>
         </is>
       </c>
     </row>
@@ -1207,12 +1207,12 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Backend models</t>
+          <t>Backend API</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>backend/app/models/agent_run.py</t>
+          <t>backend/app/api/ws.py</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>SQLAlchemy ORM / enums — the DB schema.</t>
+          <t>FastAPI routes.</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>backend/app/models/app_setting.py</t>
+          <t>backend/app/models/__init__.py</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>backend/app/models/artifact.py</t>
+          <t>backend/app/models/agent_run.py</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>backend/app/models/audit_event.py</t>
+          <t>backend/app/models/app_setting.py</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>backend/app/models/enums.py</t>
+          <t>backend/app/models/artifact.py</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>backend/app/models/gate.py</t>
+          <t>backend/app/models/audit_event.py</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>backend/app/models/push_queue.py</t>
+          <t>backend/app/models/enums.py</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>backend/app/models/story.py</t>
+          <t>backend/app/models/flaky_signature.py</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1407,12 +1407,12 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Backend schemas</t>
+          <t>Backend models</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>backend/app/schemas/__init__.py</t>
+          <t>backend/app/models/gate.py</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Pydantic API request/response models.</t>
+          <t>SQLAlchemy ORM / enums — the DB schema.</t>
         </is>
       </c>
     </row>
@@ -1432,12 +1432,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Backend agents core</t>
+          <t>Backend models</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/agents/__init__.py</t>
+          <t>backend/app/models/push_queue.py</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Agent registry, engine, schemas, prompt loader, demo fixtures.</t>
+          <t>SQLAlchemy ORM / enums — the DB schema.</t>
         </is>
       </c>
     </row>
@@ -1457,12 +1457,12 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Backend agents core</t>
+          <t>Backend models</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/agents/demo_outputs.py</t>
+          <t>backend/app/models/release.py</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Agent registry, engine, schemas, prompt loader, demo fixtures.</t>
+          <t>SQLAlchemy ORM / enums — the DB schema.</t>
         </is>
       </c>
     </row>
@@ -1482,12 +1482,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Backend agents core</t>
+          <t>Backend models</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/agents/engine.py</t>
+          <t>backend/app/models/risk_acceptance.py</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Agent registry, engine, schemas, prompt loader, demo fixtures.</t>
+          <t>SQLAlchemy ORM / enums — the DB schema.</t>
         </is>
       </c>
     </row>
@@ -1507,12 +1507,12 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Backend agents core</t>
+          <t>Backend models</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/agents/output_schemas.py</t>
+          <t>backend/app/models/story.py</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Agent registry, engine, schemas, prompt loader, demo fixtures.</t>
+          <t>SQLAlchemy ORM / enums — the DB schema.</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Backend agents core</t>
+          <t>Backend schemas</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/agents/prompts.py</t>
+          <t>backend/app/schemas/__init__.py</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Agent registry, engine, schemas, prompt loader, demo fixtures.</t>
+          <t>Pydantic API request/response models.</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/agents/registry.py</t>
+          <t>backend/app/services/agents/__init__.py</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -1582,12 +1582,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Backend services</t>
+          <t>Backend agents core</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/__init__.py</t>
+          <t>backend/app/services/agents/demo_outputs.py</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
+          <t>Agent registry, engine, schemas, prompt loader, demo fixtures.</t>
         </is>
       </c>
     </row>
@@ -1607,12 +1607,12 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Backend services</t>
+          <t>Backend agents core</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/agent_health.py</t>
+          <t>backend/app/services/agents/engine.py</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
+          <t>Agent registry, engine, schemas, prompt loader, demo fixtures.</t>
         </is>
       </c>
     </row>
@@ -1632,12 +1632,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Backend services</t>
+          <t>Backend agents core</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/artifacts/__init__.py</t>
+          <t>backend/app/services/agents/output_schemas.py</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
+          <t>Agent registry, engine, schemas, prompt loader, demo fixtures.</t>
         </is>
       </c>
     </row>
@@ -1657,12 +1657,12 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Backend services</t>
+          <t>Backend agents core</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/artifacts/parsers.py</t>
+          <t>backend/app/services/agents/prompts.py</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
+          <t>Agent registry, engine, schemas, prompt loader, demo fixtures.</t>
         </is>
       </c>
     </row>
@@ -1682,12 +1682,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Backend services</t>
+          <t>Backend agents core</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/artifacts/service.py</t>
+          <t>backend/app/services/agents/registry.py</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
+          <t>Agent registry, engine, schemas, prompt loader, demo fixtures.</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/audit.py</t>
+          <t>backend/app/services/__init__.py</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/challenger.py</t>
+          <t>backend/app/services/agent_health.py</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/copado/__init__.py</t>
+          <t>backend/app/services/artifacts/__init__.py</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/copado/fixtures.py</t>
+          <t>backend/app/services/artifacts/parsers.py</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/copado/normaliser.py</t>
+          <t>backend/app/services/artifacts/service.py</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/copado/service.py</t>
+          <t>backend/app/services/audit.py</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/evals.py</t>
+          <t>backend/app/services/challenger.py</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/evidence_pack.py</t>
+          <t>backend/app/services/copado/__init__.py</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/feedback.py</t>
+          <t>backend/app/services/copado/fixtures.py</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/github/__init__.py</t>
+          <t>backend/app/services/copado/normaliser.py</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/github/adapter.py</t>
+          <t>backend/app/services/copado/service.py</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/github/factory.py</t>
+          <t>backend/app/services/evals.py</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -2012,7 +2012,7 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/github/mock_adapter.py</t>
+          <t>backend/app/services/evidence_pack.py</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/github/rest_adapter.py</t>
+          <t>backend/app/services/feedback.py</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/github/service.py</t>
+          <t>backend/app/services/flaky_intel.py</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/__init__.py</t>
+          <t>backend/app/services/github/__init__.py</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/adapter.py</t>
+          <t>backend/app/services/github/adapter.py</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/adf.py</t>
+          <t>backend/app/services/github/factory.py</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/factory.py</t>
+          <t>backend/app/services/github/mock_adapter.py</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/field_mapping.py</t>
+          <t>backend/app/services/github/rest_adapter.py</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/mock_adapter.py</t>
+          <t>backend/app/services/github/service.py</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/push_service.py</t>
+          <t>backend/app/services/jira/__init__.py</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/rest_adapter.py</t>
+          <t>backend/app/services/jira/adapter.py</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/jira/sync_service.py</t>
+          <t>backend/app/services/jira/adf.py</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/pipeline_view.py</t>
+          <t>backend/app/services/jira/factory.py</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/referee.py</t>
+          <t>backend/app/services/jira/field_mapping.py</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/replay.py</t>
+          <t>backend/app/services/jira/mock_adapter.py</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/scheduler.py</t>
+          <t>backend/app/services/jira/push_service.py</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/settings_service.py</t>
+          <t>backend/app/services/jira/rest_adapter.py</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/work_service.py</t>
+          <t>backend/app/services/jira/sync_service.py</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>backend/app/services/workflow.py</t>
+          <t>backend/app/services/pipeline_view.py</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>backend/app/services/ws.py</t>
+          <t>backend/app/services/referee.py</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -2507,12 +2507,12 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/ac_compliance/v1.md</t>
+          <t>backend/app/services/replay.py</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2532,12 +2532,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/ac_compliance/v2.md</t>
+          <t>backend/app/services/reporting.py</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2557,12 +2557,12 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/ac_compliance/v3.md</t>
+          <t>backend/app/services/risk_register.py</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2582,12 +2582,12 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/apex_coverage/v1.md</t>
+          <t>backend/app/services/scheduler.py</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2607,12 +2607,12 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/apex_coverage/v2.md</t>
+          <t>backend/app/services/settings_service.py</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2632,12 +2632,12 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/apex_coverage/v3.md</t>
+          <t>backend/app/services/work_service.py</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2657,12 +2657,12 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/bdd_generator/v1.md</t>
+          <t>backend/app/services/workflow.py</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2682,12 +2682,12 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Agent prompts</t>
+          <t>Backend services</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/bdd_generator/v2.md</t>
+          <t>backend/app/services/ws.py</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
+          <t>Connectors (Jira/GitHub/Copado), referee, feedback, evidence pack, etc.</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/bdd_generator/v3.md</t>
+          <t>backend/prompts/ac_compliance/v1.md</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/bdd_generator/v4.md</t>
+          <t>backend/prompts/ac_compliance/v2.md</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
@@ -2762,7 +2762,7 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/change_management/v1.md</t>
+          <t>backend/prompts/ac_compliance/v3.md</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/change_management/v2.md</t>
+          <t>backend/prompts/apex_coverage/v1.md</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/code_review/v1.md</t>
+          <t>backend/prompts/apex_coverage/v2.md</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -2837,7 +2837,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/code_review/v2.md</t>
+          <t>backend/prompts/apex_coverage/v3.md</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/compliance_ac_advisor/v1.md</t>
+          <t>backend/prompts/bdd_generator/v1.md</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/consumer_duty_mapper/v1.md</t>
+          <t>backend/prompts/bdd_generator/v2.md</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/defect_triage/v1.md</t>
+          <t>backend/prompts/bdd_generator/v3.md</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/deployability_validation/v1.md</t>
+          <t>backend/prompts/bdd_generator/v4.md</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/deployment_risk/v1.md</t>
+          <t>backend/prompts/change_management/v1.md</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/deployment_risk/v2.md</t>
+          <t>backend/prompts/change_management/v2.md</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
@@ -3012,7 +3012,7 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/fca_regulatory_impact/v1.md</t>
+          <t>backend/prompts/code_review/v1.md</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/financial_data_integrity/v1.md</t>
+          <t>backend/prompts/code_review/v2.md</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/financial_data_integrity/v2.md</t>
+          <t>backend/prompts/compliance_ac_advisor/v1.md</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/integration_e2e_journey/v1.md</t>
+          <t>backend/prompts/consumer_duty_mapper/v1.md</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/monitoring_hypercare/v1.md</t>
+          <t>backend/prompts/defect_triage/v1.md</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/monitoring_hypercare/v2.md</t>
+          <t>backend/prompts/deployability_validation/v1.md</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/post_deploy_verification/v1.md</t>
+          <t>backend/prompts/deployment_risk/v1.md</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/regression_scope/v1.md</t>
+          <t>backend/prompts/deployment_risk/v2.md</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/regression_scope/v2.md</t>
+          <t>backend/prompts/fca_regulatory_impact/v1.md</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/regulatory_audit_trail/v1.md</t>
+          <t>backend/prompts/financial_data_integrity/v1.md</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/regulatory_audit_trail/v2.md</t>
+          <t>backend/prompts/financial_data_integrity/v2.md</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/release_notes/v1.md</t>
+          <t>backend/prompts/integration_e2e_journey/v1.md</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/release_readiness/v1.md</t>
+          <t>backend/prompts/monitoring_hypercare/v1.md</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/release_readiness/v2.md</t>
+          <t>backend/prompts/monitoring_hypercare/v2.md</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/security_dast/v1.md</t>
+          <t>backend/prompts/post_deploy_verification/v1.md</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/static_analysis/v1.md</t>
+          <t>backend/prompts/regression_scope/v1.md</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/static_analysis/v2.md</t>
+          <t>backend/prompts/regression_scope/v2.md</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/static_analysis/v3.md</t>
+          <t>backend/prompts/regulatory_audit_trail/v1.md</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/story_quality/v1.md</t>
+          <t>backend/prompts/regulatory_audit_trail/v2.md</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/test_data_management/v1.md</t>
+          <t>backend/prompts/release_notes/v1.md</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/test_execution_analyst/v1.md</t>
+          <t>backend/prompts/release_readiness/v1.md</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/test_execution_analyst/v2.md</t>
+          <t>backend/prompts/release_readiness/v2.md</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
@@ -3562,7 +3562,7 @@
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/three_amigos/v1.md</t>
+          <t>backend/prompts/security_dast/v1.md</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/three_amigos/v2.md</t>
+          <t>backend/prompts/static_analysis/v1.md</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/three_amigos/v3.md</t>
+          <t>backend/prompts/static_analysis/v2.md</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/three_amigos/v4.md</t>
+          <t>backend/prompts/static_analysis/v3.md</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/three_amigos/v5.md</t>
+          <t>backend/prompts/story_quality/v1.md</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
@@ -3687,7 +3687,7 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>backend/prompts/uat_signoff_coordinator/v1.md</t>
+          <t>backend/prompts/test_data_management/v1.md</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
@@ -3712,7 +3712,7 @@
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>backend/prompts/uat_signoff_coordinator/v2.md</t>
+          <t>backend/prompts/test_execution_analyst/v1.md</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
@@ -3732,12 +3732,12 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Eval golden data</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>backend/evals/golden/financial_data_integrity.json</t>
+          <t>backend/prompts/test_execution_analyst/v2.md</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>Expert-labelled golden cases — the test suite (and eval harness) fails without them.</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3757,12 +3757,12 @@
       </c>
       <c r="B131" s="5" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/__init__.py</t>
+          <t>backend/prompts/three_amigos/v1.md</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="E131" s="6" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3782,12 +3782,12 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/conftest.py</t>
+          <t>backend/prompts/three_amigos/v2.md</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3807,12 +3807,12 @@
       </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_api.py</t>
+          <t>backend/prompts/three_amigos/v3.md</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
@@ -3822,7 +3822,7 @@
       </c>
       <c r="E133" s="6" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3832,12 +3832,12 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_artifacts.py</t>
+          <t>backend/prompts/three_amigos/v4.md</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
@@ -3847,7 +3847,7 @@
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3857,12 +3857,12 @@
       </c>
       <c r="B135" s="5" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_audit.py</t>
+          <t>backend/prompts/three_amigos/v5.md</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
@@ -3872,7 +3872,7 @@
       </c>
       <c r="E135" s="6" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3882,12 +3882,12 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_confidence.py</t>
+          <t>backend/prompts/uat_signoff_coordinator/v1.md</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3907,12 +3907,12 @@
       </c>
       <c r="B137" s="5" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Agent prompts</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_copado.py</t>
+          <t>backend/prompts/uat_signoff_coordinator/v2.md</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
@@ -3922,7 +3922,7 @@
       </c>
       <c r="E137" s="6" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Versioned agent prompts — the AI behaviour. App fails without these.</t>
         </is>
       </c>
     </row>
@@ -3932,12 +3932,12 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Backend tests</t>
+          <t>Eval golden data</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_dev_agents.py</t>
+          <t>backend/evals/golden/financial_data_integrity.json</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>Run these to prove the migration is intact (pytest).</t>
+          <t>Expert-labelled golden cases — the test suite (and eval harness) fails without them.</t>
         </is>
       </c>
     </row>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_engine.py</t>
+          <t>backend/tests/__init__.py</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
@@ -3987,7 +3987,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_evidence_pack.py</t>
+          <t>backend/tests/conftest.py</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_feedback.py</t>
+          <t>backend/tests/test_api.py</t>
         </is>
       </c>
       <c r="D141" s="3" t="inlineStr">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_github.py</t>
+          <t>backend/tests/test_artifacts.py</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_pipeline_view.py</t>
+          <t>backend/tests/test_audit.py</t>
         </is>
       </c>
       <c r="D143" s="3" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_push.py</t>
+          <t>backend/tests/test_confidence.py</t>
         </is>
       </c>
       <c r="D144" s="3" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_referee.py</t>
+          <t>backend/tests/test_copado.py</t>
         </is>
       </c>
       <c r="D145" s="3" t="inlineStr">
@@ -4137,7 +4137,7 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_refinement_regulatory.py</t>
+          <t>backend/tests/test_dev_agents.py</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_release_agents.py</t>
+          <t>backend/tests/test_engine.py</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_replay.py</t>
+          <t>backend/tests/test_evidence_pack.py</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
@@ -4212,7 +4212,7 @@
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_rest_adapter.py</t>
+          <t>backend/tests/test_feedback.py</t>
         </is>
       </c>
       <c r="D149" s="3" t="inlineStr">
@@ -4237,7 +4237,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_settings.py</t>
+          <t>backend/tests/test_gate_rejection_recovery.py</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_severity.py</t>
+          <t>backend/tests/test_github.py</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
@@ -4287,7 +4287,7 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_skip.py</t>
+          <t>backend/tests/test_pipeline_view.py</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_sync.py</t>
+          <t>backend/tests/test_push.py</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -4337,7 +4337,7 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_testing_agents.py</t>
+          <t>backend/tests/test_quality_debt.py</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="C155" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_three_amigos_enrichment.py</t>
+          <t>backend/tests/test_referee.py</t>
         </is>
       </c>
       <c r="D155" s="3" t="inlineStr">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_traceability.py</t>
+          <t>backend/tests/test_refinement_regulatory.py</t>
         </is>
       </c>
       <c r="D156" s="3" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="C157" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_trust_services.py</t>
+          <t>backend/tests/test_release_agents.py</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -4437,7 +4437,7 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>backend/tests/test_work_queue.py</t>
+          <t>backend/tests/test_replay.py</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="C159" s="5" t="inlineStr">
         <is>
-          <t>backend/tests/test_workflow.py</t>
+          <t>backend/tests/test_reporting.py</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
@@ -4482,12 +4482,12 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Backend (other)</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>backend/pytest.ini</t>
+          <t>backend/tests/test_rest_adapter.py</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
@@ -4497,7 +4497,7 @@
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>Backend support file.</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4507,12 +4507,12 @@
       </c>
       <c r="B161" s="5" t="inlineStr">
         <is>
-          <t>Frontend deps</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C161" s="5" t="inlineStr">
         <is>
-          <t>frontend/package-lock.json</t>
+          <t>backend/tests/test_settings.py</t>
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="E161" s="6" t="inlineStr">
         <is>
-          <t>npm manifest + lockfile — reproducible install. DO migrate these.</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4532,12 +4532,12 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Frontend deps</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>frontend/package.json</t>
+          <t>backend/tests/test_severity.py</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
@@ -4547,7 +4547,7 @@
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>npm manifest + lockfile — reproducible install. DO migrate these.</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4557,12 +4557,12 @@
       </c>
       <c r="B163" s="5" t="inlineStr">
         <is>
-          <t>Frontend config</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C163" s="5" t="inlineStr">
         <is>
-          <t>frontend/index.html</t>
+          <t>backend/tests/test_skip.py</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="E163" s="6" t="inlineStr">
         <is>
-          <t>Vite/TS/Tailwind/PostCSS config + index.html.</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4582,12 +4582,12 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Frontend config</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>frontend/tsconfig.json</t>
+          <t>backend/tests/test_sync.py</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>Vite/TS/Tailwind/PostCSS config + index.html.</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4607,12 +4607,12 @@
       </c>
       <c r="B165" s="5" t="inlineStr">
         <is>
-          <t>Frontend config</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C165" s="5" t="inlineStr">
         <is>
-          <t>frontend/vite.config.ts</t>
+          <t>backend/tests/test_testing_agents.py</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
@@ -4622,7 +4622,7 @@
       </c>
       <c r="E165" s="6" t="inlineStr">
         <is>
-          <t>Vite/TS/Tailwind/PostCSS config + index.html.</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4632,12 +4632,12 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/App.tsx</t>
+          <t>backend/tests/test_three_amigos_enrichment.py</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4657,12 +4657,12 @@
       </c>
       <c r="B167" s="5" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C167" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/ErrorBoundary.tsx</t>
+          <t>backend/tests/test_traceability.py</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="E167" s="6" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4682,12 +4682,12 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/api.ts</t>
+          <t>backend/tests/test_trust_services.py</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4707,12 +4707,12 @@
       </c>
       <c r="B169" s="5" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C169" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/components/ArtifactsPanel.tsx</t>
+          <t>backend/tests/test_work_queue.py</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="E169" s="6" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4732,12 +4732,12 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend tests</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/components/AuditView.tsx</t>
+          <t>backend/tests/test_workflow.py</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -4747,7 +4747,7 @@
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Run these to prove the migration is intact (pytest).</t>
         </is>
       </c>
     </row>
@@ -4757,12 +4757,12 @@
       </c>
       <c r="B171" s="5" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Backend (other)</t>
         </is>
       </c>
       <c r="C171" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/components/GateModal.tsx</t>
+          <t>backend/pytest.ini</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
@@ -4772,7 +4772,7 @@
       </c>
       <c r="E171" s="6" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Backend support file.</t>
         </is>
       </c>
     </row>
@@ -4782,12 +4782,12 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Frontend deps</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/components/InsightsView.tsx</t>
+          <t>frontend/package-lock.json</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>npm manifest + lockfile — reproducible install. DO migrate these.</t>
         </is>
       </c>
     </row>
@@ -4807,12 +4807,12 @@
       </c>
       <c r="B173" s="5" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Frontend deps</t>
         </is>
       </c>
       <c r="C173" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/components/PipelineBoard.tsx</t>
+          <t>frontend/package.json</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="E173" s="6" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>npm manifest + lockfile — reproducible install. DO migrate these.</t>
         </is>
       </c>
     </row>
@@ -4832,12 +4832,12 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Frontend config</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/components/PipelineGraph.tsx</t>
+          <t>frontend/index.html</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Vite/TS/Tailwind/PostCSS config + index.html.</t>
         </is>
       </c>
     </row>
@@ -4857,12 +4857,12 @@
       </c>
       <c r="B175" s="5" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Frontend config</t>
         </is>
       </c>
       <c r="C175" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/components/PushQueueView.tsx</t>
+          <t>frontend/tsconfig.json</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
@@ -4872,7 +4872,7 @@
       </c>
       <c r="E175" s="6" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Vite/TS/Tailwind/PostCSS config + index.html.</t>
         </is>
       </c>
     </row>
@@ -4882,12 +4882,12 @@
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>Frontend source</t>
+          <t>Frontend config</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/components/RunCard.tsx</t>
+          <t>frontend/vite.config.ts</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>React app source (components, types, api client).</t>
+          <t>Vite/TS/Tailwind/PostCSS config + index.html.</t>
         </is>
       </c>
     </row>
@@ -4912,7 +4912,7 @@
       </c>
       <c r="C177" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/components/SettingsPage.tsx</t>
+          <t>frontend/src/App.tsx</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
@@ -4937,7 +4937,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/components/StoryDrawer.tsx</t>
+          <t>frontend/src/ErrorBoundary.tsx</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
@@ -4962,7 +4962,7 @@
       </c>
       <c r="C179" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/components/WorkQueue.tsx</t>
+          <t>frontend/src/api.ts</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/index.css</t>
+          <t>frontend/src/components/ArtifactsPanel.tsx</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
@@ -5012,7 +5012,7 @@
       </c>
       <c r="C181" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/main.tsx</t>
+          <t>frontend/src/components/AuditView.tsx</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/types.ts</t>
+          <t>frontend/src/components/GateModal.tsx</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="C183" s="5" t="inlineStr">
         <is>
-          <t>frontend/src/ui.tsx</t>
+          <t>frontend/src/components/InsightsView.tsx</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/ws.ts</t>
+          <t>frontend/src/components/PipelineBoard.tsx</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
@@ -5107,12 +5107,12 @@
       </c>
       <c r="B185" s="5" t="inlineStr">
         <is>
-          <t>Frontend (other)</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C185" s="5" t="inlineStr">
         <is>
-          <t>frontend/.gitignore</t>
+          <t>frontend/src/components/PipelineGraph.tsx</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="E185" s="6" t="inlineStr">
         <is>
-          <t>Frontend support file.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -5132,12 +5132,12 @@
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>Frontend (other)</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>frontend/tsconfig.tsbuildinfo</t>
+          <t>frontend/src/components/PushQueueView.tsx</t>
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>Frontend support file.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -5157,22 +5157,22 @@
       </c>
       <c r="B187" s="5" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C187" s="5" t="inlineStr">
         <is>
-          <t>README.md</t>
-        </is>
-      </c>
-      <c r="D187" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/components/ReportsView.tsx</t>
+        </is>
+      </c>
+      <c r="D187" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E187" s="6" t="inlineStr">
         <is>
-          <t>Setup + overview. Read before running setup.ps1.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -5182,22 +5182,22 @@
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>docs/COPADO-INTEGRATION.md</t>
-        </is>
-      </c>
-      <c r="D188" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/components/RiskRegisterView.tsx</t>
+        </is>
+      </c>
+      <c r="D188" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -5207,22 +5207,22 @@
       </c>
       <c r="B189" s="5" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C189" s="5" t="inlineStr">
         <is>
-          <t>docs/File-Manifest.xlsx</t>
-        </is>
-      </c>
-      <c r="D189" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/components/RunCard.tsx</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E189" s="6" t="inlineStr">
         <is>
-          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -5232,22 +5232,22 @@
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>docs/MIGRATION-FILES.xlsx</t>
-        </is>
-      </c>
-      <c r="D190" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/components/SettingsPage.tsx</t>
+        </is>
+      </c>
+      <c r="D190" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -5257,22 +5257,22 @@
       </c>
       <c r="B191" s="5" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C191" s="5" t="inlineStr">
         <is>
-          <t>docs/RESTRICTED-LAPTOP.md</t>
-        </is>
-      </c>
-      <c r="D191" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/components/StoryDrawer.tsx</t>
+        </is>
+      </c>
+      <c r="D191" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E191" s="6" t="inlineStr">
         <is>
-          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -5282,22 +5282,22 @@
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>docs/ROADMAP.md</t>
-        </is>
-      </c>
-      <c r="D192" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/components/WorkQueue.tsx</t>
+        </is>
+      </c>
+      <c r="D192" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -5307,22 +5307,22 @@
       </c>
       <c r="B193" s="5" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Frontend source</t>
         </is>
       </c>
       <c r="C193" s="5" t="inlineStr">
         <is>
-          <t>docs/SEVERITY.md</t>
-        </is>
-      </c>
-      <c r="D193" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
+          <t>frontend/src/index.css</t>
+        </is>
+      </c>
+      <c r="D193" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
       <c r="E193" s="6" t="inlineStr">
         <is>
-          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+          <t>React app source (components, types, api client).</t>
         </is>
       </c>
     </row>
@@ -5332,27 +5332,377 @@
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
+          <t>Frontend source</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>frontend/src/main.tsx</t>
+        </is>
+      </c>
+      <c r="D194" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E194" s="4" t="inlineStr">
+        <is>
+          <t>React app source (components, types, api client).</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="5" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" s="5" t="inlineStr">
+        <is>
+          <t>Frontend source</t>
+        </is>
+      </c>
+      <c r="C195" s="5" t="inlineStr">
+        <is>
+          <t>frontend/src/types.ts</t>
+        </is>
+      </c>
+      <c r="D195" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E195" s="6" t="inlineStr">
+        <is>
+          <t>React app source (components, types, api client).</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>Frontend source</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>frontend/src/ui.tsx</t>
+        </is>
+      </c>
+      <c r="D196" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E196" s="4" t="inlineStr">
+        <is>
+          <t>React app source (components, types, api client).</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="5" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" s="5" t="inlineStr">
+        <is>
+          <t>Frontend source</t>
+        </is>
+      </c>
+      <c r="C197" s="5" t="inlineStr">
+        <is>
+          <t>frontend/src/ws.ts</t>
+        </is>
+      </c>
+      <c r="D197" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E197" s="6" t="inlineStr">
+        <is>
+          <t>React app source (components, types, api client).</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>Frontend (other)</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>frontend/.gitignore</t>
+        </is>
+      </c>
+      <c r="D198" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E198" s="4" t="inlineStr">
+        <is>
+          <t>Frontend support file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="5" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" s="5" t="inlineStr">
+        <is>
+          <t>Frontend (other)</t>
+        </is>
+      </c>
+      <c r="C199" s="5" t="inlineStr">
+        <is>
+          <t>frontend/tsconfig.tsbuildinfo</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E199" s="6" t="inlineStr">
+        <is>
+          <t>Frontend support file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="C194" s="2" t="inlineStr">
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+      <c r="D200" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E200" s="4" t="inlineStr">
+        <is>
+          <t>Setup + overview. Read before running setup.ps1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" s="5" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C201" s="5" t="inlineStr">
+        <is>
+          <t>docs/COPADO-INTEGRATION.md</t>
+        </is>
+      </c>
+      <c r="D201" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E201" s="6" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>docs/File-Manifest.xlsx</t>
+        </is>
+      </c>
+      <c r="D202" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E202" s="4" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="5" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" s="5" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C203" s="5" t="inlineStr">
+        <is>
+          <t>docs/MIGRATION-FILES-CONTENT.txt</t>
+        </is>
+      </c>
+      <c r="D203" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E203" s="6" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>docs/MIGRATION-FILES.xlsx</t>
+        </is>
+      </c>
+      <c r="D204" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E204" s="4" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="5" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" s="5" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C205" s="5" t="inlineStr">
+        <is>
+          <t>docs/RESTRICTED-LAPTOP.md</t>
+        </is>
+      </c>
+      <c r="D205" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E205" s="6" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>docs/ROADMAP.md</t>
+        </is>
+      </c>
+      <c r="D206" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E206" s="4" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="5" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" s="5" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C207" s="5" t="inlineStr">
+        <is>
+          <t>docs/SEVERITY.md</t>
+        </is>
+      </c>
+      <c r="D207" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="E207" s="6" t="inlineStr">
+        <is>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
         <is>
           <t>docs/Typing-Checklist.xlsx</t>
         </is>
       </c>
-      <c r="D194" s="7" t="inlineStr">
+      <c r="D208" s="7" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="E194" s="4" t="inlineStr">
+      <c r="E208" s="4" t="inlineStr">
         <is>
           <t>Design/spec docs. Not needed to run, needed to understand.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E194"/>
+  <autoFilter ref="A1:E208"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: refresh migration manifest (206 tracked files)
Reflects the gitignore cleanup: tsconfig.tsbuildinfo (build cache)
dropped from the tracked set — it is regenerable, not migratable.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MIGRATION-FILES.xlsx
+++ b/docs/MIGRATION-FILES.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Rebuild steps" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Files to migrate'!$A$1:$E$208</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Files to migrate'!$A$1:$E$207</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E208"/>
+  <dimension ref="A1:E207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5457,22 +5457,22 @@
       </c>
       <c r="B199" s="5" t="inlineStr">
         <is>
-          <t>Frontend (other)</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="C199" s="5" t="inlineStr">
         <is>
-          <t>frontend/tsconfig.tsbuildinfo</t>
-        </is>
-      </c>
-      <c r="D199" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>README.md</t>
+        </is>
+      </c>
+      <c r="D199" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
         </is>
       </c>
       <c r="E199" s="6" t="inlineStr">
         <is>
-          <t>Frontend support file.</t>
+          <t>Setup + overview. Read before running setup.ps1.</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>docs/COPADO-INTEGRATION.md</t>
         </is>
       </c>
       <c r="D200" s="7" t="inlineStr">
@@ -5497,7 +5497,7 @@
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>Setup + overview. Read before running setup.ps1.</t>
+          <t>Design/spec docs. Not needed to run, needed to understand.</t>
         </is>
       </c>
     </row>
@@ -5512,7 +5512,7 @@
       </c>
       <c r="C201" s="5" t="inlineStr">
         <is>
-          <t>docs/COPADO-INTEGRATION.md</t>
+          <t>docs/File-Manifest.xlsx</t>
         </is>
       </c>
       <c r="D201" s="7" t="inlineStr">
@@ -5537,7 +5537,7 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>docs/File-Manifest.xlsx</t>
+          <t>docs/MIGRATION-FILES-CONTENT.txt</t>
         </is>
       </c>
       <c r="D202" s="7" t="inlineStr">
@@ -5562,7 +5562,7 @@
       </c>
       <c r="C203" s="5" t="inlineStr">
         <is>
-          <t>docs/MIGRATION-FILES-CONTENT.txt</t>
+          <t>docs/MIGRATION-FILES.xlsx</t>
         </is>
       </c>
       <c r="D203" s="7" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>docs/MIGRATION-FILES.xlsx</t>
+          <t>docs/RESTRICTED-LAPTOP.md</t>
         </is>
       </c>
       <c r="D204" s="7" t="inlineStr">
@@ -5612,7 +5612,7 @@
       </c>
       <c r="C205" s="5" t="inlineStr">
         <is>
-          <t>docs/RESTRICTED-LAPTOP.md</t>
+          <t>docs/ROADMAP.md</t>
         </is>
       </c>
       <c r="D205" s="7" t="inlineStr">
@@ -5637,7 +5637,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>docs/ROADMAP.md</t>
+          <t>docs/SEVERITY.md</t>
         </is>
       </c>
       <c r="D206" s="7" t="inlineStr">
@@ -5662,7 +5662,7 @@
       </c>
       <c r="C207" s="5" t="inlineStr">
         <is>
-          <t>docs/SEVERITY.md</t>
+          <t>docs/Typing-Checklist.xlsx</t>
         </is>
       </c>
       <c r="D207" s="7" t="inlineStr">
@@ -5676,33 +5676,8 @@
         </is>
       </c>
     </row>
-    <row r="208">
-      <c r="A208" s="2" t="n">
-        <v>207</v>
-      </c>
-      <c r="B208" s="2" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="C208" s="2" t="inlineStr">
-        <is>
-          <t>docs/Typing-Checklist.xlsx</t>
-        </is>
-      </c>
-      <c r="D208" s="7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
-      <c r="E208" s="4" t="inlineStr">
-        <is>
-          <t>Design/spec docs. Not needed to run, needed to understand.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E208"/>
+  <autoFilter ref="A1:E207"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>